<commit_message>
Replace out-of-stock slide switches in BOM
</commit_message>
<xml_diff>
--- a/Documentation/Working_Documents/Chatterbox_BOM.xlsx
+++ b/Documentation/Working_Documents/Chatterbox_BOM.xlsx
@@ -1433,7 +1433,7 @@
       <c r="M16" s="68" t="n"/>
       <c r="N16" s="74" t="inlineStr">
         <is>
-          <t>https://www.digikey.ca/en/products/detail/c-k/os102011ma1qs1/1981431</t>
+          <t>https://www.digikey.ca/en/products/detail/c-k/os102011ma1qn1/1981430</t>
         </is>
       </c>
     </row>
@@ -1993,7 +1993,7 @@
       <c r="M28" s="68" t="n"/>
       <c r="N28" s="74" t="inlineStr">
         <is>
-          <t>https://www.digikey.ca/en/products/detail/c-k/os103011ma7qp1/1981432</t>
+          <t>https://www.digikey.ca/en/products/detail/c-k/os103011ma7qp1c/10063872</t>
         </is>
       </c>
     </row>

</xml_diff>